<commit_message>
Update MASST dataset files with improved column names
Rename columns in MASST_Dataset.csv and MASST_Dataset.xlsx, and update the MASST_1774115946873.DAT file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 73283557-eec7-4d48-b902-e46eece83672
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 6c3bbe8b-3369-49d9-b78d-d895431adb4b
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/MASST_Dataset.xlsx
+++ b/MASST_Dataset.xlsx
@@ -100,13 +100,13 @@
     <t>V27_RationingNecessary</t>
   </si>
   <si>
-    <t>V28_ConservingSavesMonney</t>
+    <t>V28_ConservingSavesMoney</t>
   </si>
   <si>
     <t>V29_NaturalGasDoneEnough</t>
   </si>
   <si>
-    <t>V30_BillSameNomatter</t>
+    <t>V30_BillSameNoMatter</t>
   </si>
   <si>
     <t>V31_CitizenCannotHelp</t>

</xml_diff>